<commit_message>
Replace the physician anesthesia case log with the corrected instructions
The September 23 template no longer tells applicants to complete separate Adult Anesthesia and Pediatric Anesthesia tabs.

Co-authored-by: gorin-research-repo <gorin-research-repo@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/case-logs/ANESTHESIA_(PHYSICIAN)_CASE_LOG_TEMPLATE_Sept_23_2026.xlsx
+++ b/case-logs/ANESTHESIA_(PHYSICIAN)_CASE_LOG_TEMPLATE_Sept_23_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\DOP Revamp\Case Log Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9349F356-410D-42F1-8269-73D54C003049}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95BA92CA-FA98-4B0F-87C4-932F7DF9BE92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2400" yWindow="2400" windowWidth="21600" windowHeight="12630" activeTab="2" xr2:uid="{A2D48BC0-44BC-4FBF-8BA7-2031E65295F7}"/>
+    <workbookView xWindow="2400" yWindow="2400" windowWidth="21600" windowHeight="12630" xr2:uid="{A2D48BC0-44BC-4FBF-8BA7-2031E65295F7}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -326,7 +326,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>104775</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="8296275" cy="4507772"/>
+    <xdr:ext cx="8296275" cy="3976666"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="2" name="TextBox 1">
@@ -341,7 +341,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="95250" y="104775"/>
-          <a:ext cx="8296275" cy="4507772"/>
+          <a:ext cx="8296275" cy="3976666"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -457,23 +457,6 @@
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
             <a:t>during the 12-month period immediately preceding the date of submission of the credentialing application. </a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-US" sz="1200" b="0" u="none">
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200" b="0" u="none">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Complete the appropriate sections (tabs) of the workbook corresponding to the privilege categories being requested (e.g., Adult Anesthesia, Pediatric Anesthesia).</a:t>
           </a:r>
         </a:p>
         <a:p>

</xml_diff>

<commit_message>
Split physician anesthesia certification lines and correct the case log
Show board certification, board eligibility, ACLS, and PeRLS on separate lines. Replace the physician case-log template with the corrected September 23 file, whose instructions no longer refer to Adult Anesthesia and Pediatric Anesthesia tabs.
</commit_message>
<xml_diff>
--- a/case-logs/ANESTHESIA_(PHYSICIAN)_CASE_LOG_TEMPLATE_Sept_23_2026.xlsx
+++ b/case-logs/ANESTHESIA_(PHYSICIAN)_CASE_LOG_TEMPLATE_Sept_23_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\DOP Revamp\Case Log Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9349F356-410D-42F1-8269-73D54C003049}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95BA92CA-FA98-4B0F-87C4-932F7DF9BE92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2400" yWindow="2400" windowWidth="21600" windowHeight="12630" activeTab="2" xr2:uid="{A2D48BC0-44BC-4FBF-8BA7-2031E65295F7}"/>
+    <workbookView xWindow="2400" yWindow="2400" windowWidth="21600" windowHeight="12630" xr2:uid="{A2D48BC0-44BC-4FBF-8BA7-2031E65295F7}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -326,7 +326,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>104775</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="8296275" cy="4507772"/>
+    <xdr:ext cx="8296275" cy="3976666"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="2" name="TextBox 1">
@@ -341,7 +341,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="95250" y="104775"/>
-          <a:ext cx="8296275" cy="4507772"/>
+          <a:ext cx="8296275" cy="3976666"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -457,23 +457,6 @@
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
             <a:t>during the 12-month period immediately preceding the date of submission of the credentialing application. </a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-US" sz="1200" b="0" u="none">
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200" b="0" u="none">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Complete the appropriate sections (tabs) of the workbook corresponding to the privilege categories being requested (e.g., Adult Anesthesia, Pediatric Anesthesia).</a:t>
           </a:r>
         </a:p>
         <a:p>

</xml_diff>